<commit_message>
Incorporar presupuestos verificados en la base
</commit_message>
<xml_diff>
--- a/Lista_Investigaciones_ECAP_RS.xlsx
+++ b/Lista_Investigaciones_ECAP_RS.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Becarios" sheetId="1" r:id="R31cf68a153d74dde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apoyo_para_Investigaciones" sheetId="2" r:id="R7d68317dbe624326"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos_Investigación" sheetId="3" r:id="Rd78c3caf17074d4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Otros_Estudios_Referenciados" sheetId="4" r:id="R9483681581694339"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Otras_Investigac_Ámbito_Estudio" sheetId="7" r:id="Ra6684ed5449d4443"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados_líneas_investigación" sheetId="5" r:id="R012fdf64078440f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados_Sistemas_ACH" sheetId="6" r:id="Rf3267eeb1f384ef0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="8" r:id="R49fcb67428a44d96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base_mapa" sheetId="9" r:id="R40646b15f5b34e3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Becarios" sheetId="1" r:id="R5828e94e1cd94474"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apoyo_para_Investigaciones" sheetId="2" r:id="Rec77cc2d42df4328"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Proyectos_Investigación" sheetId="3" r:id="Rfde16ed8ceb14cc3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Otros_Estudios_Referenciados" sheetId="4" r:id="Rac3627c29109438b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Otras_Investigac_Ámbito_Estudio" sheetId="7" r:id="R2a643be706364750"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados_líneas_investigación" sheetId="5" r:id="Re7900badc8114293"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados_Sistemas_ACH" sheetId="6" r:id="R9e5a0828a1f9430e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoja1" sheetId="8" r:id="Rd19ef5b278b84dde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base_mapa" sheetId="9" r:id="R268f25229cdc4fc9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4646,9 +4646,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="2">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="0.0000000"/>
     <x:numFmt numFmtId="201" formatCode="$#,##0.00"/>
+    <x:numFmt numFmtId="202" formatCode="&quot;$&quot;#,##0.00"/>
   </x:numFmts>
   <x:fonts count="19">
     <x:font>
@@ -5163,7 +5164,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="286">
+  <x:cellXfs count="287">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="top"/>
@@ -6006,6 +6007,9 @@
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="201" fontId="17" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="17" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
@@ -16386,7 +16390,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb2d5c6dbe7af47ef"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1e44703e32934045"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -16416,7 +16420,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re0101d4a072f49a2"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra1a642e2557747e3"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -16446,7 +16450,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4808ec86363b41d0"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc1b7c126dd4a4ab7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -16481,7 +16485,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf9b7ab0d916f440e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc0ba0d9dc1764189"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -16511,7 +16515,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb107b9e36afa43ba"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R170972f1b93d4f2b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -16541,7 +16545,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9db7fe03257f4186"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0fdcf2192ee04175"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -16571,7 +16575,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb78155a213a041b5"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R4be999589a5d4175"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -16601,7 +16605,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re2dfe0c2316f4d90"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R79d95a077ef8430b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -16631,7 +16635,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd5d4ba27084047cb"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re1e7207106e04c5b"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -22090,37 +22094,37 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="R03cc5a5019e94e02"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="Rde7fa7f0e70e483e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="Rb300926c7b244a09"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="R7e49cff108664f04"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="Rf4a10410d5444055"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="Rf677fb0a8a534bf8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="R0db58135ca11489e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="R55030d5a1eca4342"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="Rf32e55dbff914adb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="R5f53cb8ae7c54d23"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="R292a056c126c46f1"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="R41487ba230ee4230"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="R75f467f08a594c13"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="R51fb59cdf04d4531"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="R0ba3891923c5499a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="R6f44178869be4e7c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="R6db01ddd4068463e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="Ra016ba3e71754f94"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="R18a8739dc3b84766"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="R9b948a400fa44b60"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="Rbeb11823cb5849c5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="R57f80bc8a61c4636"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="Rf5202083d2e648a0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="R66a1d52b57104afb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="R5cdfeae573684deb"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="R8cbe5224903d423c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="R186c53ed73ef460a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="R681ca5327e6c4325"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="R18c8c007bfca4bd5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="Raa937b79c2db4b83"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="Rc5206c7572c8447b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="R73c77af1655b4714"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="Rf9b398b299634060"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="R4559d5d55ec8461a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="Rc786670f3feb4420"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="R196c03befae04231"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="R893bed6c11204a2a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="R4f179fd2b83749df"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="Rb2d218155e0d4fea"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="R1da5c077490b4725"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="R491f71f06f124ff9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="Rf2d2401ecddb4d82"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="R37bbffea11c34951"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="Rb73d7939ce5b4214"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="Ra3d3c623bdac48cb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="Ra8d470febaf64d10"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="Rf2d733d53f2b456e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="Rbfc81c9010614c29"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="R82dab3c32279496f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="Reba8f5f6cde84230"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="Re851e714254d4676"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="R27d6d5770b604202"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78cf26111bc74f6a"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5495ad6dfbd64b5a"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22ab0ef5f7a744ac"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra2088302c06148ed"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26601,41 +26605,41 @@
     <x:mergeCell ref="A55:B55"/>
   </x:mergeCells>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="R82761e29ba82466a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="R31b5f6b562044c28"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="R278e104aad7d4c88"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="R55b0884b747a4d61"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="R8c4fa3bcaecb4839"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="R141e47abd7c14284"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="Rf1097bd8b3244eb9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="R3917bef26d1b476c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="Rbf48e9c273194b03"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="R3db19c67168a4324"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="R71bc1337e8624649"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="Rab4acb205b144d7c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="R9047d3ec0d11486f"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="R28ab6a4235cf4531"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R653dee8af0ca458e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="R806ad4c7a89144f3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="R9b73dd32bf3e4182"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="R0fc9e5af8eaa4519"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="R220519ce4ce04faa"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="R0ce65737e85943ac"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="R5859323d3a55457a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="Rc9d7dc81a3ec427a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="Rd1d3b4796e2f4f2a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="R1e0dba9dea724207"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="R231aadb2cb28478c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="R6faa742561904cac"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="Rc204e7b4131440d4"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="R47436e04782f4b78"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="R70a078d18e7148ca"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="R9f3e9236b35f48a9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="Rb13b4dd214da4ccf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="R6cf5d25d099147a8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="Rde2371ba14d4477b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="R10dd388f8f34499f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="R8c4ae95af31247d8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="R4c6c8443e92744b5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="R8d3937b2a89345eb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="R4efb570548de4694"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="Re8be03f12e3842e9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="R667efd3709e442a4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="Ree5b383bd310445a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="Ra7cf3a6dde24484e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="R242a2abd36e64963"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="R774582d8ff4a4240"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R8327113f38724da0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="R6ad4b171f4964f6f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="R176ccd83dcbf43cc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="R0e4a5a70a62e475d"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="R44b4f5af7b8f4c26"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="Rb6f48cb53b1341b7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="R64ae526ea15740f7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="Rd890411ae0f54faf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="Rcdf564b4cf1e4850"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="Rf4ca61076f2143ba"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="Rdab12017c06f48f0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="Rc285f7de7761418b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="Ref7f6abbb92649e3"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="R2f0543b9614c4dd9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="R7eaa25fca01a4f3a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="R93d8618035484510"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9446c90f7ace43aa"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabe8b32de933459a"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbe2fdae2d4b4af1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9238d79fd6744238"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -33564,7 +33568,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R657b35cd54ed410e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9237785fc13b4944"/>
 </x:worksheet>
 </file>
 
@@ -34761,7 +34765,7 @@
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e80111e6a684ebd"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9966594efda24252"/>
 </x:worksheet>
 </file>
 
@@ -36231,7 +36235,9 @@
       <x:c r="I39" s="276" t="str">
         <x:v>El estudio estableció un protocolo in vitro para Draba obovata orientado a la restauración ecológica en el Área de Conservación Hídrica Antisana. Probó tratamientos de desinfección, germinación y regulación de crecimiento en medio MS. El uso de detergente al 2 %, etanol al 70 % e hipoclorito de sodio al 2,5 % evitó contaminación y oxidación; el medio MS con sacarosa logró 86,67 % de germinación y BAP más AIA promovió la mayor proliferación de brotes.</x:v>
       </x:c>
-      <x:c r="J39" s="284"/>
+      <x:c r="J39" s="286" t="n">
+        <x:v>1500</x:v>
+      </x:c>
     </x:row>
     <x:row r="40" ht="88" customHeight="1">
       <x:c r="A40" s="276" t="str">
@@ -36899,7 +36905,9 @@
       <x:c r="I61" s="276" t="str">
         <x:v>La investigación caracteriza el agente asociado a la pudrición radicular de Calamagrostis fibrovaginata en el páramo de Antisana. Trabaja con aislamientos de plantas afectadas, cultivos en PDA, microscopía, amplificación de ITS, β-tubulina y TEF1-α, filogenia de máxima verosimilitud y ensayos de patogenicidad. El documento disponible identifica el aislado dentro del complejo Fusarium sambucinum y reporta que indujo síntomas de pudrición y marchitez en condiciones controladas; la delimitación a nivel de especie requiere marcadores adicionales.</x:v>
       </x:c>
-      <x:c r="J61" s="284"/>
+      <x:c r="J61" s="286" t="n">
+        <x:v>1650.6</x:v>
+      </x:c>
     </x:row>
     <x:row r="62" ht="88" customHeight="1">
       <x:c r="A62" s="276" t="str">
@@ -36929,7 +36937,9 @@
       <x:c r="I62" s="276" t="str">
         <x:v>El estudio analiza la cadena de valor de plantas nativas en los viveros comunitarios Las Tolas y San Francisco de Cruz Loma. Con un diseño mixto, observacional y transversal para datos de 2025, integra entrevistas, observación, registros administrativos, mapeo de flujos, cálculo de costos y comparación con un vivero comercial. El documento disponible identifica dependencia de un solo comprador y precios de venta de 0,50 USD inferiores al precio mínimo viable estimado de 0,71 a 0,88 USD por planta, y propone acciones 5W2H y B2B para fortalecer la sostenibilidad.</x:v>
       </x:c>
-      <x:c r="J62" s="284"/>
+      <x:c r="J62" s="286" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="63" ht="88" customHeight="1">
       <x:c r="A63" s="276" t="str">
@@ -37023,7 +37033,9 @@
       <x:c r="I65" s="276" t="str">
         <x:v>El estudio analizó la concentración y distribución de parámetros físico-químicos en el embalse Salve Faccha, reservorio altoandino que aporta agua al abastecimiento de Quito. Combinó datos históricos, una hidroboya multiparamétrica y muestreos mensuales, con climogramas Walter-Lieth, rosas de viento, mapas de calor e isolíneas verticales. Identificó estratificaciones térmicas leves a 2,75 y 7,50 m y químicas entre 5 y 10 m en la época relativamente seca, influenciadas por el viento, sin anoxia ni estratificación marcada.</x:v>
       </x:c>
-      <x:c r="J65" s="284"/>
+      <x:c r="J65" s="286" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="66" ht="88" customHeight="1">
       <x:c r="A66" s="276" t="str">
@@ -37085,7 +37097,9 @@
       <x:c r="I67" s="276" t="str">
         <x:v>Analizó la sostenibilidad del modelo comunitario de agua potable de Yunguilla desde las dimensiones técnica, económica, sociocultural y ambiental. Combinó entrevistas, encuestas a hogares, observación, cartografía social y grupos focales, sistematizados con una matriz de cuádruple resultado. Encontró una organización comunitaria consolidada e infraestructura funcional, pero también deterioro de tuberías y válvulas, turbidez estacional, dependencia de un técnico y ausencia de fondo de emergencia; plantea reforzar mantenimiento, relevo técnico y gestión financiera.</x:v>
       </x:c>
-      <x:c r="J67" s="284"/>
+      <x:c r="J67" s="286" t="n">
+        <x:v>2000</x:v>
+      </x:c>
     </x:row>
     <x:row r="68" ht="88" customHeight="1">
       <x:c r="A68" s="276" t="str">
@@ -37243,7 +37257,9 @@
       <x:c r="I72" s="276" t="str">
         <x:v>Caracterizó la morfometría de la cuenca Rumipamba en las laderas del Pichincha para describir su comportamiento físico e hidrológico. Delimitó el área, instaló nueve puntos de control y realizó un vuelo con dron de más de 5.000 imágenes para generar un modelo digital de elevación y ortomosaico; después calculó parámetros en QGIS y SAGA GIS. La cuenca, de 577 ha, presentó forma alargada, pendiente media de 37,9° y densidad de drenaje de 2,2 km/km², rasgos compatibles con escorrentía rápida y erosión.</x:v>
       </x:c>
-      <x:c r="J72" s="284"/>
+      <x:c r="J72" s="286" t="n">
+        <x:v>3086</x:v>
+      </x:c>
     </x:row>
     <x:row r="73" ht="88" customHeight="1">
       <x:c r="A73" s="276" t="str">
@@ -37273,7 +37289,9 @@
       <x:c r="I73" s="276" t="str">
         <x:v>Cuantificó y caracterizó microplásticos en agua superficial y sedimentos de cinco lagos altoandinos del sistema Papallacta–Oyacachi. Analizó abundancia, tamaño, color, forma y composición polimérica, además de posibles fuentes locales y atmosféricas. Registró microplásticos en ambos medios, con predominio de fibras y películas y presencia de celofán, polietileno y polipropileno; el estudio plantea que pesca, campismo, senderismo y transporte atmosférico podrían contribuir a los aportes.</x:v>
       </x:c>
-      <x:c r="J73" s="284"/>
+      <x:c r="J73" s="286" t="n">
+        <x:v>1738.93</x:v>
+      </x:c>
     </x:row>
     <x:row r="74" ht="88" customHeight="1">
       <x:c r="A74" s="276" t="str">
@@ -37397,7 +37415,9 @@
       <x:c r="I77" s="276" t="str">
         <x:v>Determinó la variación espacio-temporal del área superficial de humedales altoandinos y su relación con la morfología de cuencas del sistema Ñucanchi Turubamba, Papallacta–Oyacachi. Procesó imágenes Sentinel-1 en Google Earth Engine con clasificación Otsu, calculó área inundada y frecuencia de inundación, y aplicó análisis de componentes principales y agrupamiento. La extensión inundada varió entre 0,6 % y 42,6 % de las cuencas, con un máximo en mayo, y se identificaron tres grupos con dinámicas diferenciadas.</x:v>
       </x:c>
-      <x:c r="J77" s="284"/>
+      <x:c r="J77" s="286" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="78" ht="88" customHeight="1">
       <x:c r="A78" s="276" t="str">
@@ -37619,7 +37639,9 @@
       <x:c r="I84" s="276" t="str">
         <x:v>Evaluó cuatro tratamientos de sustrato para propagar esquejes de Polylepis incana en el vivero de Ponce Paluguillo como apoyo a la restauración. Comparó mezclas de tierra negra, tierra de páramo, hojarasca y cascajo mediante propiedades físico-químicas, densidad, nutrientes y respuesta de las plántulas. Los tratamientos no difirieron en pH, conductividad, potencial redox ni cenizas, pero sí en densidad, nitrógeno y fósforo; el informe destaca la importancia de porosidad, baja compactación y materia orgánica para el establecimiento inicial.</x:v>
       </x:c>
-      <x:c r="J84" s="284"/>
+      <x:c r="J84" s="286" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="85" ht="88" customHeight="1">
       <x:c r="A85" s="276" t="str">
@@ -37681,7 +37703,9 @@
       <x:c r="I86" s="276" t="str">
         <x:v>Evaluó la dinámica de sedimentos y el color real en los ríos Jatunhuayco y Antisana del sistema La Mica–Quito Sur. Realizó campañas de campo, aforos con micromolinete y dilución química, análisis de fracciones de sólidos, turbidez, color, pH, temperatura y oxígeno, y procesó los datos en RStudio y QGIS. Jatunhuayco presentó mayores sedimentos y variabilidad de color, mientras Antisana fue más estable, comportamiento que la fuente asocia a su origen glaciar y a aportes de ojos de agua.</x:v>
       </x:c>
-      <x:c r="J86" s="284"/>
+      <x:c r="J86" s="286" t="n">
+        <x:v>2107.48</x:v>
+      </x:c>
     </x:row>
     <x:row r="87" ht="88" customHeight="1">
       <x:c r="A87" s="276" t="str">
@@ -37839,7 +37863,9 @@
       <x:c r="I91" s="276" t="str">
         <x:v>Analizó la relación entre factores físico-químicos y comunidades de microalgas en lagos del sistema Papallacta–Oyacachi, durante dos campañas entre 2020 y 2021. Recolectó fitoplancton y perifiton, los identificó microscópicamente y aplicó análisis de correspondencia canónica y similitud. Identificó 106 especies; lagos y reservorios tuvieron baja similitud florística, y conductividad y transparencia fueron las variables más influyentes, sin una relación mayor de nutrientes con la presencia de especies.</x:v>
       </x:c>
-      <x:c r="J91" s="284"/>
+      <x:c r="J91" s="286" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="92" ht="88" customHeight="1">
       <x:c r="A92" s="276" t="str">
@@ -37899,7 +37925,9 @@
       <x:c r="I93" s="276" t="str">
         <x:v>Mapeó dinámicamente bofedales en áreas de interés hídrico de Pichincha, Napo y Cotopaxi mediante imágenes Sentinel-1 y Sentinel-2, clasificación supervisada y un Water Cloud Model calibrado con humedad superficial in situ. Comparó cartografía óptica, radar y basada en humedad para examinar variación intra e interanual, con énfasis en Jatunhuaycu. La integración óptica-radar permitió el análisis dinámico; en 2023 se estimaron 28.972 ha de humedales y el modelo calibrado alcanzó R = 0,79, aunque subestimó área frente a la clasificación radar.</x:v>
       </x:c>
-      <x:c r="J93" s="284"/>
+      <x:c r="J93" s="286" t="n">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="94" ht="88" customHeight="1">
       <x:c r="A94" s="276" t="str">
@@ -38871,7 +38899,9 @@
       <x:c r="I125" s="276" t="str">
         <x:v>El proyecto de trazadores colorimétricos en ACHA Atacazo buscó comprender conexiones hídricas en las cuencas Dique Norte y Carachas, asociadas al predio San Gabriel. Propuso inyectar eosina y fluoresceína en dos puntos, monitorear hasta seis sitios con fluorómetros o carbón activado durante seis meses y contar con apoyo de guardapáramos. Se esperaban tiempos de tránsito, conexiones entre cabeceras, galerías y río, zonas de recarga y posibles trasvases para orientar la gestión del agua.</x:v>
       </x:c>
-      <x:c r="J125" s="284"/>
+      <x:c r="J125" s="286" t="n">
+        <x:v>4101</x:v>
+      </x:c>
     </x:row>
     <x:row r="126" ht="88" customHeight="1">
       <x:c r="A126" s="276" t="str">
@@ -39026,7 +39056,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R22a142a495db441d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99b766ec262245ac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>